<commit_message>
changing menu screen + updating algo
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
   <si>
     <t>UCD vs UCSC</t>
   </si>
@@ -43,364 +43,337 @@
     <t>Score (Winner First)</t>
   </si>
   <si>
-    <t>11:00</t>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>WD3</t>
+  </si>
+  <si>
+    <t>vs</t>
+  </si>
+  <si>
+    <t>Aditi Kavipurapu + Muyen Liang</t>
+  </si>
+  <si>
+    <t>Daphne Huang + Rhea Zou</t>
+  </si>
+  <si>
+    <t>XD2</t>
+  </si>
+  <si>
+    <t>Richard huang + Kristine Ngo</t>
+  </si>
+  <si>
+    <t>Ashton Lee + Amanda Ng</t>
+  </si>
+  <si>
+    <t>XD1</t>
+  </si>
+  <si>
+    <t>Leyang Ding + Xin Huang</t>
+  </si>
+  <si>
+    <t>Adam Tay + Tara Chou</t>
+  </si>
+  <si>
+    <t>XD3</t>
+  </si>
+  <si>
+    <t>Robert Chang  + Erika Lai</t>
+  </si>
+  <si>
+    <t>Vivan Sinha + Kristin Song</t>
+  </si>
+  <si>
+    <t>MD5</t>
+  </si>
+  <si>
+    <t>Justin Larson + Samarth Sridhara</t>
+  </si>
+  <si>
+    <t>Howard Huang + Ray Sun</t>
+  </si>
+  <si>
+    <t>XD8</t>
+  </si>
+  <si>
+    <t>Adrian Luo + Julie Ma</t>
+  </si>
+  <si>
+    <t>Rehadyan Utomo + Nadia Kho</t>
+  </si>
+  <si>
+    <t>11:15</t>
+  </si>
+  <si>
+    <t>WS1</t>
+  </si>
+  <si>
+    <t>Erika Lai</t>
+  </si>
+  <si>
+    <t>Tara Chou</t>
+  </si>
+  <si>
+    <t>MD1</t>
+  </si>
+  <si>
+    <t>Richard Huang + Jun Jie Lai</t>
+  </si>
+  <si>
+    <t>Adam Tay + Kevin Lan</t>
+  </si>
+  <si>
+    <t>XD7</t>
+  </si>
+  <si>
+    <t>Kyle Huang + Yvonne Wang</t>
+  </si>
+  <si>
+    <t>MS7</t>
+  </si>
+  <si>
+    <t>Jon Moser</t>
+  </si>
+  <si>
+    <t>Thet Paing (David) Da Na</t>
+  </si>
+  <si>
+    <t>WD6</t>
+  </si>
+  <si>
+    <t>Anni Zhang + Elaine Jiang</t>
+  </si>
+  <si>
+    <t>WS4</t>
+  </si>
+  <si>
+    <t>Elaine Tsou</t>
+  </si>
+  <si>
+    <t>Anjuli Oey</t>
+  </si>
+  <si>
+    <t>12:00</t>
+  </si>
+  <si>
+    <t>MS2</t>
+  </si>
+  <si>
+    <t>Leyang Ding</t>
+  </si>
+  <si>
+    <t>Brad Chiu</t>
+  </si>
+  <si>
+    <t>MD3</t>
+  </si>
+  <si>
+    <t>Jon Moser + Kyle Fang</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Ryan Zhu</t>
+  </si>
+  <si>
+    <t>XD6</t>
+  </si>
+  <si>
+    <t>Andy Li + Muyen</t>
+  </si>
+  <si>
+    <t>Warren Chang + Ashley Zheng</t>
+  </si>
+  <si>
+    <t>XD4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claudia Xu + Andrew Yeow </t>
+  </si>
+  <si>
+    <t>Kevin Lan + Eileen Pan</t>
+  </si>
+  <si>
+    <t>MD9</t>
+  </si>
+  <si>
+    <t>Junru Su + Aaron Lim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leo Chen + Jackie Dai </t>
+  </si>
+  <si>
+    <t>MS4</t>
+  </si>
+  <si>
+    <t>Neil Patel</t>
+  </si>
+  <si>
+    <t>Ray Sun</t>
+  </si>
+  <si>
+    <t>12:45</t>
+  </si>
+  <si>
+    <t>WD1</t>
+  </si>
+  <si>
+    <t>Joy Yang + Xin Huang</t>
+  </si>
+  <si>
+    <t>Amanda Ng + Tara Chou</t>
+  </si>
+  <si>
+    <t>MS3</t>
+  </si>
+  <si>
+    <t>Robert Chang</t>
+  </si>
+  <si>
+    <t>Ryan Zhu</t>
+  </si>
+  <si>
+    <t>MS1</t>
+  </si>
+  <si>
+    <t>Jun Jie Lai</t>
+  </si>
+  <si>
+    <t>Patrick Chi</t>
+  </si>
+  <si>
+    <t>MD11</t>
+  </si>
+  <si>
+    <t>Rehadyan Utomo + Warren Chang</t>
+  </si>
+  <si>
+    <t>WD5</t>
+  </si>
+  <si>
+    <t>Claudia Xu + Erika Lai</t>
+  </si>
+  <si>
+    <t>Sarah Gao + Fiona Chen</t>
+  </si>
+  <si>
+    <t>MD4</t>
+  </si>
+  <si>
+    <t>Vo Ly + Brandon Leung</t>
+  </si>
+  <si>
+    <t>Cameron Kato + Harsh Srivastav</t>
+  </si>
+  <si>
+    <t>01:30</t>
+  </si>
+  <si>
+    <t>WS2</t>
+  </si>
+  <si>
+    <t>Joy Yang</t>
+  </si>
+  <si>
+    <t>Ashley Huang</t>
   </si>
   <si>
     <t>WS3</t>
   </si>
   <si>
-    <t>vs</t>
-  </si>
-  <si>
-    <t>Cindy Shing</t>
-  </si>
-  <si>
-    <t>Natasha Kulkarni</t>
-  </si>
-  <si>
-    <t>XD3</t>
-  </si>
-  <si>
-    <t>Claudia Xu + Jeremy Leung</t>
-  </si>
-  <si>
-    <t>Brian Huang + Amy Sha</t>
-  </si>
-  <si>
-    <t>MD1</t>
-  </si>
-  <si>
-    <t>Richard Huang + Robert Chang</t>
-  </si>
-  <si>
-    <t>Brian Huang + Sam Lai</t>
-  </si>
-  <si>
-    <t>WS4</t>
-  </si>
-  <si>
-    <t>Xin Huang</t>
-  </si>
-  <si>
-    <t>Jenny Lei</t>
-  </si>
-  <si>
-    <t>WD3</t>
-  </si>
-  <si>
-    <t>Aysia Saeturn + Diana Del Rosario</t>
-  </si>
-  <si>
-    <t>Emily Lam + Jennifer Kim</t>
-  </si>
-  <si>
-    <t>MD5</t>
-  </si>
-  <si>
-    <t>Adrian Lam + Jon Moser</t>
-  </si>
-  <si>
-    <t>Yash Malegaonkar + Nathan Nguyen</t>
-  </si>
-  <si>
-    <t>11:30</t>
+    <t>Kristine Ngo</t>
+  </si>
+  <si>
+    <t>Rosamund Li</t>
+  </si>
+  <si>
+    <t>MS6</t>
+  </si>
+  <si>
+    <t>Kyle Fang</t>
+  </si>
+  <si>
+    <t>Brandon Wu</t>
+  </si>
+  <si>
+    <t>MD10</t>
+  </si>
+  <si>
+    <t>Neil Patel + Andrew Yeow</t>
+  </si>
+  <si>
+    <t>Arav Sachdeva + Aarav Singh</t>
+  </si>
+  <si>
+    <t>MD6</t>
+  </si>
+  <si>
+    <t>Jonathan Li + Sean Tan</t>
+  </si>
+  <si>
+    <t>Edwin Tang + Jonathon Cheng</t>
+  </si>
+  <si>
+    <t>MD2</t>
+  </si>
+  <si>
+    <t>Leyang Ding + Robert Chang</t>
+  </si>
+  <si>
+    <t>Ashton Lee + Vivan Sinha</t>
+  </si>
+  <si>
+    <t>02:15</t>
+  </si>
+  <si>
+    <t>MS5</t>
+  </si>
+  <si>
+    <t>Andrew Yeow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jackie Dai </t>
   </si>
   <si>
     <t>WD2</t>
   </si>
   <si>
-    <t>Iris Lee + Claudia Xu</t>
-  </si>
-  <si>
-    <t>Natasha Kulkarni + Vara Madem</t>
-  </si>
-  <si>
-    <t>WD1</t>
-  </si>
-  <si>
-    <t>Xin Huang + Steffi Ling</t>
-  </si>
-  <si>
-    <t>Sarah Chun + Hannah Wang</t>
-  </si>
-  <si>
-    <t>MD3</t>
-  </si>
-  <si>
-    <t>Sidney Wang + Bo Yan</t>
-  </si>
-  <si>
-    <t>Allan Sun + Suneet Katrekar</t>
-  </si>
-  <si>
-    <t>XD7</t>
-  </si>
-  <si>
-    <t>Joey Mai + Geoffrey Ku</t>
-  </si>
-  <si>
-    <t>Akhilesh Nidamanuri + Jennifer Kim</t>
-  </si>
-  <si>
-    <t>MD2</t>
-  </si>
-  <si>
-    <t>Kevin Cuan + Jeremy Leung</t>
-  </si>
-  <si>
-    <t>Eric Wang + Brandon Wang</t>
-  </si>
-  <si>
-    <t>MS9</t>
-  </si>
-  <si>
-    <t>Ethan Chen</t>
-  </si>
-  <si>
-    <t>Nathan Mei</t>
-  </si>
-  <si>
-    <t>12:00</t>
-  </si>
-  <si>
-    <t>WD5</t>
-  </si>
-  <si>
-    <t>Jenny Lei + Iris Chan</t>
-  </si>
-  <si>
-    <t>MS3</t>
-  </si>
-  <si>
-    <t>Justin Liu</t>
-  </si>
-  <si>
-    <t>Evan Chen</t>
-  </si>
-  <si>
-    <t>WS2</t>
-  </si>
-  <si>
-    <t>Joy Yang</t>
-  </si>
-  <si>
-    <t>Sarah Chun</t>
-  </si>
-  <si>
-    <t>MD10</t>
-  </si>
-  <si>
-    <t>Ethan Chan + Anthony Ngo</t>
-  </si>
-  <si>
-    <t>Curtis Luu + Akhilesh Nidamanuri</t>
-  </si>
-  <si>
-    <t>MS11</t>
-  </si>
-  <si>
-    <t>Robert Chang</t>
-  </si>
-  <si>
-    <t>Yash Malegaonkar</t>
+    <t>Ashley Huang + Kristin Song</t>
   </si>
   <si>
     <t>WD4</t>
   </si>
   <si>
-    <t>Joey Mai + Amie Zheng</t>
-  </si>
-  <si>
-    <t>Dorothy Li + Hazel Chen</t>
-  </si>
-  <si>
-    <t>12:30</t>
-  </si>
-  <si>
-    <t>MS2</t>
-  </si>
-  <si>
-    <t>Allan Sun</t>
-  </si>
-  <si>
-    <t>MD6</t>
-  </si>
-  <si>
-    <t>Geoffrey Ku + Vo Ly</t>
-  </si>
-  <si>
-    <t>Andrew Ryu + Nathan Mei</t>
-  </si>
-  <si>
-    <t>WS1</t>
-  </si>
-  <si>
-    <t>Amy Sha</t>
-  </si>
-  <si>
-    <t>XD1</t>
-  </si>
-  <si>
-    <t>Robert Chang + Xin Huang</t>
-  </si>
-  <si>
-    <t>Evan Chen + Sarah Chun</t>
+    <t>Julie La + Khanh Tran</t>
+  </si>
+  <si>
+    <t>Eileen Pan + Alicia Wang</t>
   </si>
   <si>
     <t>MD8</t>
   </si>
   <si>
-    <t>Adam Vu  + Justin Yi</t>
-  </si>
-  <si>
-    <t>XD8</t>
-  </si>
-  <si>
-    <t>Richard Huang + Amber Zhang</t>
-  </si>
-  <si>
-    <t>William Wu + Jenny Lei</t>
-  </si>
-  <si>
-    <t>01:00</t>
-  </si>
-  <si>
-    <t>WS5</t>
-  </si>
-  <si>
-    <t>Dorothy Li</t>
-  </si>
-  <si>
-    <t>XD2</t>
-  </si>
-  <si>
-    <t>Steffi Ling + Kevin Cuan</t>
-  </si>
-  <si>
-    <t>Sam Lai + Hannah Wang</t>
+    <t>Andy Li + Jason Wu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anton Luu + Justin Wang </t>
+  </si>
+  <si>
+    <t>XD5</t>
+  </si>
+  <si>
+    <t>Aditi Kavipurapu + Ken Sibal</t>
+  </si>
+  <si>
+    <t>Randy Huang + Rhea Zou</t>
   </si>
   <si>
     <t>MD7</t>
   </si>
   <si>
-    <t>Shak Guruswami + Dustin Wang</t>
-  </si>
-  <si>
-    <t>MS12</t>
-  </si>
-  <si>
-    <t>Nathan Nguyen</t>
-  </si>
-  <si>
-    <t>XD5</t>
-  </si>
-  <si>
-    <t>Stephanie Lau + Anthony Ngo</t>
-  </si>
-  <si>
-    <t>Brandon Wang + Natasha Kulkarni</t>
-  </si>
-  <si>
-    <t>MS7</t>
-  </si>
-  <si>
-    <t>Ethan Chan</t>
-  </si>
-  <si>
-    <t>Aidan Au Yeung</t>
-  </si>
-  <si>
-    <t>01:30</t>
-  </si>
-  <si>
-    <t>XD6</t>
-  </si>
-  <si>
-    <t>Collette Shu + Ethan Chen</t>
-  </si>
-  <si>
-    <t>Shak Guruswami + Vara Madem</t>
-  </si>
-  <si>
-    <t>MS1</t>
-  </si>
-  <si>
-    <t>Kevin Cuan</t>
-  </si>
-  <si>
-    <t>Sam Lai</t>
-  </si>
-  <si>
-    <t>MS5</t>
-  </si>
-  <si>
-    <t>Jon Moser</t>
-  </si>
-  <si>
-    <t>Anish Bansel</t>
-  </si>
-  <si>
-    <t>MD4</t>
-  </si>
-  <si>
-    <t>MS10</t>
-  </si>
-  <si>
-    <t>Nathan Yu</t>
-  </si>
-  <si>
-    <t>MS8</t>
-  </si>
-  <si>
-    <t>Jeff Cheung</t>
-  </si>
-  <si>
-    <t>Andrew Ryu</t>
-  </si>
-  <si>
-    <t>02:00</t>
-  </si>
-  <si>
-    <t>XD4</t>
-  </si>
-  <si>
-    <t>Joy Yang + Justin Liu</t>
-  </si>
-  <si>
-    <t>Curtis Luu  + Emily Lam</t>
-  </si>
-  <si>
-    <t>XD10</t>
-  </si>
-  <si>
-    <t>MD9</t>
-  </si>
-  <si>
-    <t>Bruce Bai + Van Ly</t>
-  </si>
-  <si>
-    <t>XD9</t>
-  </si>
-  <si>
-    <t>Julius Chang + Dorothy Li</t>
-  </si>
-  <si>
-    <t>MS4</t>
-  </si>
-  <si>
-    <t>Neil Patel</t>
-  </si>
-  <si>
-    <t>Eric Wang</t>
-  </si>
-  <si>
-    <t>MS6</t>
-  </si>
-  <si>
-    <t>Sidney Wang</t>
-  </si>
-  <si>
-    <t>Suneet Katrekar</t>
+    <t>Bill Wong + Donald Ly</t>
+  </si>
+  <si>
+    <t>Evan Wang + Brandon Wu</t>
   </si>
   <si>
     <t>A-Team Tally</t>
@@ -852,7 +825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="15.7109375" customWidth="1"/>
@@ -896,7 +869,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="3" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="M2" s="3"/>
     </row>
@@ -913,11 +886,11 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="4">
-        <f>SUM( L6, L7, L8, L10, L12, L13, L14, L16, L19, L20, L24, L26, L27, L31, L37)</f>
+        <f>SUM( L6, L7, L8, L9, L12, L13, L18, L19, L24, L25, L26, L30, L31, L35, L37)</f>
         <v>0</v>
       </c>
       <c r="M3" s="4">
-        <f>SUM( M6, M7, M8, M10, M12, M13, M14, M16, M19, M20, M24, M26, M27, M31, M37)</f>
+        <f>SUM( M6, M7, M8, M9, M12, M13, M18, M19, M24, M25, M26, M30, M31, M35, M37)</f>
         <v>0</v>
       </c>
     </row>
@@ -934,7 +907,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="3" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="M4" s="3"/>
     </row>
@@ -967,11 +940,11 @@
       </c>
       <c r="K5" s="5"/>
       <c r="L5" s="4">
-        <f>SUM( L6, L7, L8, L9, L10, L11, L12, L13, L14, L15, L16, L17, L18, L19, L20, L21, L22, L23, L24, L25, L26, L27, L28, L29, L30, L31, L32, L33, L34, L35, L36, L37, L38, L39, L40, L41, L42, L43, L44, L45, L46, L47)</f>
+        <f>SUM( L6, L7, L8, L9, L10, L11, L12, L13, L14, L15, L16, L17, L18, L19, L20, L21, L22, L23, L24, L25, L26, L27, L28, L29, L30, L31, L32, L33, L34, L35, L36, L37, L38, L39, L40, L41)</f>
         <v>0</v>
       </c>
       <c r="M5" s="4">
-        <f>SUM( M6, M7, M8, M9, M10, M11, M12, M13, M14, M15, M16, M17, M18, M19, M20, M21, M22, M23, M24, M25, M26, M27, M28, M29, M30, M31, M32, M33, M34, M35, M36, M37, M38, M39, M40, M41, M42, M43, M44, M45, M46, M47)</f>
+        <f>SUM( M6, M7, M8, M9, M10, M11, M12, M13, M14, M15, M16, M17, M18, M19, M20, M21, M22, M23, M24, M25, M26, M27, M28, M29, M30, M31, M32, M33, M34, M35, M36, M37, M38, M39, M40, M41)</f>
         <v>0</v>
       </c>
     </row>
@@ -1221,14 +1194,14 @@
         <v>36</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I14" s="6"/>
       <c r="J14" s="7"/>
@@ -1247,17 +1220,17 @@
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="7"/>
@@ -1276,17 +1249,17 @@
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I16" s="6"/>
       <c r="J16" s="7"/>
@@ -1305,17 +1278,17 @@
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="7"/>
@@ -1329,24 +1302,24 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B18" s="6">
         <v>1</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" s="7"/>
@@ -1365,17 +1338,17 @@
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="7"/>
@@ -1394,17 +1367,17 @@
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>55</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I20" s="6"/>
       <c r="J20" s="7"/>
@@ -1423,17 +1396,17 @@
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="7"/>
@@ -1452,17 +1425,17 @@
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I22" s="6"/>
       <c r="J22" s="7"/>
@@ -1481,17 +1454,17 @@
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="7"/>
@@ -1505,17 +1478,17 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B24" s="6">
         <v>1</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="5" t="s">
@@ -1573,14 +1546,14 @@
         <v>72</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>21</v>
+        <v>73</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I26" s="6"/>
       <c r="J26" s="7"/>
@@ -1599,10 +1572,10 @@
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
@@ -1631,14 +1604,14 @@
         <v>77</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I28" s="6"/>
       <c r="J28" s="7"/>
@@ -1657,17 +1630,17 @@
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I29" s="6"/>
       <c r="J29" s="7"/>
@@ -1681,24 +1654,24 @@
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B30" s="6">
         <v>1</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I30" s="6"/>
       <c r="J30" s="7"/>
@@ -1717,17 +1690,17 @@
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="7"/>
@@ -1746,17 +1719,17 @@
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>18</v>
+        <v>91</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="I32" s="6"/>
       <c r="J32" s="7"/>
@@ -1775,17 +1748,17 @@
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I33" s="6"/>
       <c r="J33" s="7"/>
@@ -1804,17 +1777,17 @@
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="7"/>
@@ -1833,17 +1806,17 @@
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="7"/>
@@ -1857,24 +1830,24 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B36" s="6">
         <v>1</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I36" s="6"/>
       <c r="J36" s="7"/>
@@ -1893,17 +1866,17 @@
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="7" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I37" s="6"/>
       <c r="J37" s="7"/>
@@ -1922,17 +1895,17 @@
       </c>
       <c r="C38" s="7"/>
       <c r="D38" s="7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I38" s="6"/>
       <c r="J38" s="7"/>
@@ -1951,17 +1924,17 @@
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
       <c r="I39" s="6"/>
       <c r="J39" s="7"/>
@@ -1980,17 +1953,17 @@
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="I40" s="6"/>
       <c r="J40" s="7"/>
@@ -2009,17 +1982,17 @@
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="7" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="I41" s="6"/>
       <c r="J41" s="7"/>
@@ -2031,184 +2004,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
-      <c r="A42" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B42" s="6">
-        <v>1</v>
-      </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="F42" s="6"/>
-      <c r="G42" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="I42" s="6"/>
-      <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
-      <c r="L42" s="6">
-        <v>1</v>
-      </c>
-      <c r="M42" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="5"/>
-      <c r="B43" s="6">
-        <v>2</v>
-      </c>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F43" s="6"/>
-      <c r="G43" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H43" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="I43" s="6"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="6">
-        <v>1</v>
-      </c>
-      <c r="M43" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13">
-      <c r="A44" s="5"/>
-      <c r="B44" s="6">
-        <v>3</v>
-      </c>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F44" s="6"/>
-      <c r="G44" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="I44" s="6"/>
-      <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
-      <c r="L44" s="6">
-        <v>1</v>
-      </c>
-      <c r="M44" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13">
-      <c r="A45" s="5"/>
-      <c r="B45" s="6">
-        <v>4</v>
-      </c>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F45" s="6"/>
-      <c r="G45" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="I45" s="6"/>
-      <c r="J45" s="7"/>
-      <c r="K45" s="7"/>
-      <c r="L45" s="6">
-        <v>1</v>
-      </c>
-      <c r="M45" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13">
-      <c r="A46" s="5"/>
-      <c r="B46" s="6">
-        <v>5</v>
-      </c>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="F46" s="6"/>
-      <c r="G46" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="I46" s="6"/>
-      <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
-      <c r="L46" s="6">
-        <v>1</v>
-      </c>
-      <c r="M46" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13">
-      <c r="A47" s="5"/>
-      <c r="B47" s="6">
-        <v>6</v>
-      </c>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="F47" s="6"/>
-      <c r="G47" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H47" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="I47" s="6"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
-      <c r="L47" s="6">
-        <v>1</v>
-      </c>
-      <c r="M47" s="6">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="139">
+  <mergeCells count="120">
     <mergeCell ref="A1:K4"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="H5:I5"/>
@@ -2327,25 +2124,6 @@
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="J41:K41"/>
-    <mergeCell ref="A42:A47"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="J44:K44"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="J47:K47"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="L4:M4"/>
   </mergeCells>

</xml_diff>

<commit_message>
Updated Terminal System + Added new conflict_checker.py
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="170">
   <si>
     <t>UCD vs UCSC</t>
   </si>
@@ -43,28 +43,427 @@
     <t>Score (Winner First)</t>
   </si>
   <si>
-    <t>10:30</t>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>WD1</t>
+  </si>
+  <si>
+    <t>vs</t>
+  </si>
+  <si>
+    <t>Xin Huang + Betty Yang</t>
+  </si>
+  <si>
+    <t>Reanne Chan + Ariel Shan</t>
+  </si>
+  <si>
+    <t>MS1</t>
+  </si>
+  <si>
+    <t>Leyang Ding</t>
+  </si>
+  <si>
+    <t>Adam Tay</t>
+  </si>
+  <si>
+    <t>WS1</t>
+  </si>
+  <si>
+    <t>Jamie Yip</t>
+  </si>
+  <si>
+    <t>Ziyi Huang</t>
+  </si>
+  <si>
+    <t>WD5</t>
+  </si>
+  <si>
+    <t>Winnie Wu + Mallika Chou</t>
+  </si>
+  <si>
+    <t>Anni Zhang + Phoebe Shen</t>
+  </si>
+  <si>
+    <t>WS2</t>
+  </si>
+  <si>
+    <t>Carolyn Suryapermana</t>
+  </si>
+  <si>
+    <t>Emily Qian</t>
+  </si>
+  <si>
+    <t>MD6</t>
+  </si>
+  <si>
+    <t>Sean Tan + Kevin Cuan</t>
+  </si>
+  <si>
+    <t>Kelsey Lin + Jansen Mok</t>
+  </si>
+  <si>
+    <t>10:45</t>
+  </si>
+  <si>
+    <t>WD2</t>
+  </si>
+  <si>
+    <t>Kristine Ngo + Erika Lai</t>
+  </si>
+  <si>
+    <t>Kaylee Wang + Kristin Song</t>
+  </si>
+  <si>
+    <t>MS4</t>
+  </si>
+  <si>
+    <t>Geoffray Lee</t>
+  </si>
+  <si>
+    <t>Zheng Zhou</t>
+  </si>
+  <si>
+    <t>WS3</t>
+  </si>
+  <si>
+    <t>Chonticha Phanphanit</t>
+  </si>
+  <si>
+    <t>Chaemin Lee</t>
   </si>
   <si>
     <t>WD3</t>
   </si>
   <si>
-    <t>vs</t>
-  </si>
-  <si>
-    <t>Aditi Kavipurapu + Muyen Liang</t>
-  </si>
-  <si>
-    <t>Daphne Huang + Rhea Zou</t>
+    <t>Muyen Liang + Jamie Yip</t>
+  </si>
+  <si>
+    <t>Clarissa Chen + Yuhe Lin</t>
+  </si>
+  <si>
+    <t>MD3</t>
+  </si>
+  <si>
+    <t>Jon Moser + Jonathan Li</t>
+  </si>
+  <si>
+    <t>Aarav Rathi + Shengkai Jiang</t>
+  </si>
+  <si>
+    <t>MD11</t>
+  </si>
+  <si>
+    <t>Ryan Lei + Adrian Luu</t>
+  </si>
+  <si>
+    <t>Zevin Bansal + Vinayak Prathikanti</t>
+  </si>
+  <si>
+    <t>11:30</t>
+  </si>
+  <si>
+    <t>MD4</t>
+  </si>
+  <si>
+    <t>Sidney Wang + Adrian Luo</t>
+  </si>
+  <si>
+    <t>XD8</t>
+  </si>
+  <si>
+    <t>Ryan Lei + Jamie Yip</t>
+  </si>
+  <si>
+    <t>Kelsey Lin + Trinity Nguyen</t>
+  </si>
+  <si>
+    <t>MS8</t>
+  </si>
+  <si>
+    <t>Jonathan Li</t>
+  </si>
+  <si>
+    <t>Ryan Zhu</t>
+  </si>
+  <si>
+    <t>MD9</t>
+  </si>
+  <si>
+    <t>Jordon Kwong + Chimnay</t>
+  </si>
+  <si>
+    <t>Kyle Huang + Khai Ho</t>
+  </si>
+  <si>
+    <t>XD9</t>
+  </si>
+  <si>
+    <t>Adrian Li + Isabella Li</t>
+  </si>
+  <si>
+    <t>Howard Huang + Rosamund Li</t>
+  </si>
+  <si>
+    <t>MD1</t>
+  </si>
+  <si>
+    <t>Leyang Ding + Richard Huang</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Jason Arya</t>
+  </si>
+  <si>
+    <t>12:15</t>
+  </si>
+  <si>
+    <t>XD10</t>
+  </si>
+  <si>
+    <t>Richard Huang + Livia Rice</t>
+  </si>
+  <si>
+    <t>Jeff Chen + Stephanie Kuang</t>
+  </si>
+  <si>
+    <t>MD13</t>
+  </si>
+  <si>
+    <t>Marc Ethan Saguiped + Donnovan Saelee</t>
+  </si>
+  <si>
+    <t>Wesley Tan + Jansen Mok</t>
+  </si>
+  <si>
+    <t>MS14</t>
+  </si>
+  <si>
+    <t>Bill Wong</t>
+  </si>
+  <si>
+    <t>Jack Chu</t>
+  </si>
+  <si>
+    <t>MS11</t>
+  </si>
+  <si>
+    <t>Adrian Li</t>
+  </si>
+  <si>
+    <t>Arav Sachdeva</t>
+  </si>
+  <si>
+    <t>MD2</t>
+  </si>
+  <si>
+    <t>Benson Ngai + Geoffray Lee</t>
+  </si>
+  <si>
+    <t>Ashley Huang + Natalie Chi</t>
+  </si>
+  <si>
+    <t>XD14</t>
+  </si>
+  <si>
+    <t>Jerry Qiu + Suhani Shokeen</t>
+  </si>
+  <si>
+    <t>Haoran Qu + Janina Schieneman</t>
+  </si>
+  <si>
+    <t>01:00</t>
+  </si>
+  <si>
+    <t>MD5</t>
+  </si>
+  <si>
+    <t>Mariano Elizondo + Jerry Qiu</t>
+  </si>
+  <si>
+    <t>Jonathan Pan + Harry Zhang</t>
+  </si>
+  <si>
+    <t>MS15</t>
+  </si>
+  <si>
+    <t>Finn</t>
+  </si>
+  <si>
+    <t>Arion Togelang</t>
+  </si>
+  <si>
+    <t>XD11</t>
+  </si>
+  <si>
+    <t>Aaron Lim + Gaby Solei</t>
+  </si>
+  <si>
+    <t>Howie Liang + Angel Yeung</t>
+  </si>
+  <si>
+    <t>MS6</t>
+  </si>
+  <si>
+    <t>Adrian Luo</t>
+  </si>
+  <si>
+    <t>Jason Arya</t>
+  </si>
+  <si>
+    <t>XD13</t>
+  </si>
+  <si>
+    <t>Booker Brown + Chonticha Phanphanit</t>
+  </si>
+  <si>
+    <t>Ajay Sharma + Zinong Wang</t>
   </si>
   <si>
     <t>XD2</t>
   </si>
   <si>
-    <t>Richard huang + Kristine Ngo</t>
-  </si>
-  <si>
-    <t>Ashton Lee + Amanda Ng</t>
+    <t>Benson Ngai + Kristine Ngo</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Natalie Chi</t>
+  </si>
+  <si>
+    <t>01:45</t>
+  </si>
+  <si>
+    <t>XD7</t>
+  </si>
+  <si>
+    <t>Jonathan Li + Ehong Ng</t>
+  </si>
+  <si>
+    <t>Aarav Rathi + Jane Dong</t>
+  </si>
+  <si>
+    <t>MS16</t>
+  </si>
+  <si>
+    <t>Booker Brown</t>
+  </si>
+  <si>
+    <t>Kwanghyun Kim</t>
+  </si>
+  <si>
+    <t>XD12</t>
+  </si>
+  <si>
+    <t>Daniel Lin + Carolyn Surypermana</t>
+  </si>
+  <si>
+    <t>Vinayak Prathikanti + Caitlin Tong</t>
+  </si>
+  <si>
+    <t>MD12</t>
+  </si>
+  <si>
+    <t>Josh Luo + Karthik Villavan</t>
+  </si>
+  <si>
+    <t>Justin Wang + Anton Luu</t>
+  </si>
+  <si>
+    <t>WD4</t>
+  </si>
+  <si>
+    <t>Livia Rice + Isabella Li</t>
+  </si>
+  <si>
+    <t>Angelina Wang + Janina Schieneman</t>
+  </si>
+  <si>
+    <t>MS13</t>
+  </si>
+  <si>
+    <t>Michael Salim</t>
+  </si>
+  <si>
+    <t>Joon Choi</t>
+  </si>
+  <si>
+    <t>02:30</t>
+  </si>
+  <si>
+    <t>MD7</t>
+  </si>
+  <si>
+    <t>Aaron Lim + Bill Wong</t>
+  </si>
+  <si>
+    <t>Jonathan Pan + Jeff Chen</t>
+  </si>
+  <si>
+    <t>XD6</t>
+  </si>
+  <si>
+    <t>Adam Dinh + Minh Nguyen</t>
+  </si>
+  <si>
+    <t>Shengkai Jiang + Kristin Song</t>
+  </si>
+  <si>
+    <t>XD3</t>
+  </si>
+  <si>
+    <t>Kevin Cuan + Iris Lee</t>
+  </si>
+  <si>
+    <t>Ashton Lee + Ashley Huang</t>
+  </si>
+  <si>
+    <t>XD4</t>
+  </si>
+  <si>
+    <t>Richard Huang + Erika Lai</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Kaylee Wang</t>
+  </si>
+  <si>
+    <t>MD8</t>
+  </si>
+  <si>
+    <t>Daniel Lin + Yawei He</t>
+  </si>
+  <si>
+    <t>Arav Sachdeva + Arun Yadavalli</t>
+  </si>
+  <si>
+    <t>MD10</t>
+  </si>
+  <si>
+    <t>Michael Salim + Kyle Kimura</t>
+  </si>
+  <si>
+    <t>Howard Huang + Cameron Kato</t>
+  </si>
+  <si>
+    <t>03:15</t>
+  </si>
+  <si>
+    <t>MS7</t>
+  </si>
+  <si>
+    <t>Sidney Wang</t>
+  </si>
+  <si>
+    <t>MS10</t>
+  </si>
+  <si>
+    <t>Aaron Lim</t>
+  </si>
+  <si>
+    <t>Jake Kim</t>
+  </si>
+  <si>
+    <t>MS5</t>
+  </si>
+  <si>
+    <t>Jon Moser</t>
   </si>
   <si>
     <t>XD1</t>
@@ -73,307 +472,52 @@
     <t>Leyang Ding + Xin Huang</t>
   </si>
   <si>
-    <t>Adam Tay + Tara Chou</t>
-  </si>
-  <si>
-    <t>XD3</t>
-  </si>
-  <si>
-    <t>Robert Chang  + Erika Lai</t>
-  </si>
-  <si>
-    <t>Vivan Sinha + Kristin Song</t>
-  </si>
-  <si>
-    <t>MD5</t>
-  </si>
-  <si>
-    <t>Justin Larson + Samarth Sridhara</t>
-  </si>
-  <si>
-    <t>Howard Huang + Ray Sun</t>
-  </si>
-  <si>
-    <t>XD8</t>
-  </si>
-  <si>
-    <t>Adrian Luo + Julie Ma</t>
-  </si>
-  <si>
-    <t>Rehadyan Utomo + Nadia Kho</t>
-  </si>
-  <si>
-    <t>11:15</t>
-  </si>
-  <si>
-    <t>WS1</t>
-  </si>
-  <si>
-    <t>Erika Lai</t>
-  </si>
-  <si>
-    <t>Tara Chou</t>
-  </si>
-  <si>
-    <t>MD1</t>
-  </si>
-  <si>
-    <t>Richard Huang + Jun Jie Lai</t>
-  </si>
-  <si>
-    <t>Adam Tay + Kevin Lan</t>
-  </si>
-  <si>
-    <t>XD7</t>
-  </si>
-  <si>
-    <t>Kyle Huang + Yvonne Wang</t>
-  </si>
-  <si>
-    <t>MS7</t>
-  </si>
-  <si>
-    <t>Jon Moser</t>
-  </si>
-  <si>
-    <t>Thet Paing (David) Da Na</t>
-  </si>
-  <si>
-    <t>WD6</t>
-  </si>
-  <si>
-    <t>Anni Zhang + Elaine Jiang</t>
-  </si>
-  <si>
-    <t>WS4</t>
-  </si>
-  <si>
-    <t>Elaine Tsou</t>
-  </si>
-  <si>
-    <t>Anjuli Oey</t>
-  </si>
-  <si>
-    <t>12:00</t>
+    <t>Adam Tay + Angie Huang</t>
+  </si>
+  <si>
+    <t>MS3</t>
+  </si>
+  <si>
+    <t>Mariano Elizondo</t>
+  </si>
+  <si>
+    <t>Brad Chiu</t>
+  </si>
+  <si>
+    <t>MS9</t>
+  </si>
+  <si>
+    <t>Sean Tan</t>
+  </si>
+  <si>
+    <t>Arun Yadavalli</t>
+  </si>
+  <si>
+    <t>04:00</t>
+  </si>
+  <si>
+    <t>MS12</t>
+  </si>
+  <si>
+    <t>Kyle Kimura</t>
+  </si>
+  <si>
+    <t>Khai Ho</t>
   </si>
   <si>
     <t>MS2</t>
   </si>
   <si>
-    <t>Leyang Ding</t>
-  </si>
-  <si>
-    <t>Brad Chiu</t>
-  </si>
-  <si>
-    <t>MD3</t>
-  </si>
-  <si>
-    <t>Jon Moser + Kyle Fang</t>
-  </si>
-  <si>
-    <t>Patrick Chi + Ryan Zhu</t>
-  </si>
-  <si>
-    <t>XD6</t>
-  </si>
-  <si>
-    <t>Andy Li + Muyen</t>
-  </si>
-  <si>
-    <t>Warren Chang + Ashley Zheng</t>
-  </si>
-  <si>
-    <t>XD4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claudia Xu + Andrew Yeow </t>
-  </si>
-  <si>
-    <t>Kevin Lan + Eileen Pan</t>
-  </si>
-  <si>
-    <t>MD9</t>
-  </si>
-  <si>
-    <t>Junru Su + Aaron Lim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leo Chen + Jackie Dai </t>
-  </si>
-  <si>
-    <t>MS4</t>
-  </si>
-  <si>
-    <t>Neil Patel</t>
-  </si>
-  <si>
-    <t>Ray Sun</t>
-  </si>
-  <si>
-    <t>12:45</t>
-  </si>
-  <si>
-    <t>WD1</t>
-  </si>
-  <si>
-    <t>Joy Yang + Xin Huang</t>
-  </si>
-  <si>
-    <t>Amanda Ng + Tara Chou</t>
-  </si>
-  <si>
-    <t>MS3</t>
-  </si>
-  <si>
-    <t>Robert Chang</t>
-  </si>
-  <si>
-    <t>Ryan Zhu</t>
-  </si>
-  <si>
-    <t>MS1</t>
-  </si>
-  <si>
-    <t>Jun Jie Lai</t>
-  </si>
-  <si>
-    <t>Patrick Chi</t>
-  </si>
-  <si>
-    <t>MD11</t>
-  </si>
-  <si>
-    <t>Rehadyan Utomo + Warren Chang</t>
-  </si>
-  <si>
-    <t>WD5</t>
-  </si>
-  <si>
-    <t>Claudia Xu + Erika Lai</t>
-  </si>
-  <si>
-    <t>Sarah Gao + Fiona Chen</t>
-  </si>
-  <si>
-    <t>MD4</t>
-  </si>
-  <si>
-    <t>Vo Ly + Brandon Leung</t>
-  </si>
-  <si>
-    <t>Cameron Kato + Harsh Srivastav</t>
-  </si>
-  <si>
-    <t>01:30</t>
-  </si>
-  <si>
-    <t>WS2</t>
-  </si>
-  <si>
-    <t>Joy Yang</t>
-  </si>
-  <si>
-    <t>Ashley Huang</t>
-  </si>
-  <si>
-    <t>WS3</t>
-  </si>
-  <si>
-    <t>Kristine Ngo</t>
-  </si>
-  <si>
-    <t>Rosamund Li</t>
-  </si>
-  <si>
-    <t>MS6</t>
-  </si>
-  <si>
-    <t>Kyle Fang</t>
-  </si>
-  <si>
-    <t>Brandon Wu</t>
-  </si>
-  <si>
-    <t>MD10</t>
-  </si>
-  <si>
-    <t>Neil Patel + Andrew Yeow</t>
-  </si>
-  <si>
-    <t>Arav Sachdeva + Aarav Singh</t>
-  </si>
-  <si>
-    <t>MD6</t>
-  </si>
-  <si>
-    <t>Jonathan Li + Sean Tan</t>
-  </si>
-  <si>
-    <t>Edwin Tang + Jonathon Cheng</t>
-  </si>
-  <si>
-    <t>MD2</t>
-  </si>
-  <si>
-    <t>Leyang Ding + Robert Chang</t>
-  </si>
-  <si>
-    <t>Ashton Lee + Vivan Sinha</t>
-  </si>
-  <si>
-    <t>02:15</t>
-  </si>
-  <si>
-    <t>MS5</t>
-  </si>
-  <si>
-    <t>Andrew Yeow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jackie Dai </t>
-  </si>
-  <si>
-    <t>WD2</t>
-  </si>
-  <si>
-    <t>Ashley Huang + Kristin Song</t>
-  </si>
-  <si>
-    <t>WD4</t>
-  </si>
-  <si>
-    <t>Julie La + Khanh Tran</t>
-  </si>
-  <si>
-    <t>Eileen Pan + Alicia Wang</t>
-  </si>
-  <si>
-    <t>MD8</t>
-  </si>
-  <si>
-    <t>Andy Li + Jason Wu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anton Luu + Justin Wang </t>
+    <t>Kevin Cuan</t>
   </si>
   <si>
     <t>XD5</t>
   </si>
   <si>
-    <t>Aditi Kavipurapu + Ken Sibal</t>
-  </si>
-  <si>
-    <t>Randy Huang + Rhea Zou</t>
-  </si>
-  <si>
-    <t>MD7</t>
-  </si>
-  <si>
-    <t>Bill Wong + Donald Ly</t>
-  </si>
-  <si>
-    <t>Evan Wang + Brandon Wu</t>
+    <t>Sidney Wang + Betty Yang</t>
+  </si>
+  <si>
+    <t>Ashton Lee + Angie Huang</t>
   </si>
   <si>
     <t>A-Team Tally</t>
@@ -825,7 +969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="15.7109375" customWidth="1"/>
@@ -869,7 +1013,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="3" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="M2" s="3"/>
     </row>
@@ -886,11 +1030,11 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="4">
-        <f>SUM( L6, L7, L8, L9, L12, L13, L18, L19, L24, L25, L26, L30, L31, L35, L37)</f>
+        <f>SUM( L6, L7, L8, L10, L12, L14, L15, L16, L23, L28, L35, L44, L51, L52, L55)</f>
         <v>0</v>
       </c>
       <c r="M3" s="4">
-        <f>SUM( M6, M7, M8, M9, M12, M13, M18, M19, M24, M25, M26, M30, M31, M35, M37)</f>
+        <f>SUM( M6, M7, M8, M10, M12, M14, M15, M16, M23, M28, M35, M44, M51, M52, M55)</f>
         <v>0</v>
       </c>
     </row>
@@ -907,7 +1051,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="3" t="s">
-        <v>121</v>
+        <v>169</v>
       </c>
       <c r="M4" s="3"/>
     </row>
@@ -940,11 +1084,11 @@
       </c>
       <c r="K5" s="5"/>
       <c r="L5" s="4">
-        <f>SUM( L6, L7, L8, L9, L10, L11, L12, L13, L14, L15, L16, L17, L18, L19, L20, L21, L22, L23, L24, L25, L26, L27, L28, L29, L30, L31, L32, L33, L34, L35, L36, L37, L38, L39, L40, L41)</f>
+        <f>SUM( L6, L7, L8, L9, L10, L11, L12, L13, L14, L15, L16, L17, L18, L19, L20, L21, L22, L23, L24, L25, L26, L27, L28, L29, L30, L31, L32, L33, L34, L35, L36, L37, L38, L39, L40, L41, L42, L43, L44, L45, L46, L47, L48, L49, L50, L51, L52, L53, L54, L55, L56)</f>
         <v>0</v>
       </c>
       <c r="M5" s="4">
-        <f>SUM( M6, M7, M8, M9, M10, M11, M12, M13, M14, M15, M16, M17, M18, M19, M20, M21, M22, M23, M24, M25, M26, M27, M28, M29, M30, M31, M32, M33, M34, M35, M36, M37, M38, M39, M40, M41)</f>
+        <f>SUM( M6, M7, M8, M9, M10, M11, M12, M13, M14, M15, M16, M17, M18, M19, M20, M21, M22, M23, M24, M25, M26, M27, M28, M29, M30, M31, M32, M33, M34, M35, M36, M37, M38, M39, M40, M41, M42, M43, M44, M45, M46, M47, M48, M49, M50, M51, M52, M53, M54, M55, M56)</f>
         <v>0</v>
       </c>
     </row>
@@ -1194,14 +1338,14 @@
         <v>36</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I14" s="6"/>
       <c r="J14" s="7"/>
@@ -1220,17 +1364,17 @@
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="7"/>
@@ -1249,17 +1393,17 @@
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I16" s="6"/>
       <c r="J16" s="7"/>
@@ -1278,17 +1422,17 @@
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="7"/>
@@ -1302,24 +1446,24 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B18" s="6">
         <v>1</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" s="7"/>
@@ -1338,17 +1482,17 @@
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="7"/>
@@ -1367,17 +1511,17 @@
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I20" s="6"/>
       <c r="J20" s="7"/>
@@ -1396,17 +1540,17 @@
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="7"/>
@@ -1425,17 +1569,17 @@
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I22" s="6"/>
       <c r="J22" s="7"/>
@@ -1454,17 +1598,17 @@
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="7"/>
@@ -1478,24 +1622,24 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B24" s="6">
         <v>1</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I24" s="6"/>
       <c r="J24" s="7"/>
@@ -1514,17 +1658,17 @@
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I25" s="6"/>
       <c r="J25" s="7"/>
@@ -1543,17 +1687,17 @@
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I26" s="6"/>
       <c r="J26" s="7"/>
@@ -1572,17 +1716,17 @@
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I27" s="6"/>
       <c r="J27" s="7"/>
@@ -1601,17 +1745,17 @@
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I28" s="6"/>
       <c r="J28" s="7"/>
@@ -1630,17 +1774,17 @@
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I29" s="6"/>
       <c r="J29" s="7"/>
@@ -1654,24 +1798,24 @@
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B30" s="6">
         <v>1</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I30" s="6"/>
       <c r="J30" s="7"/>
@@ -1690,17 +1834,17 @@
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="7"/>
@@ -1719,17 +1863,17 @@
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I32" s="6"/>
       <c r="J32" s="7"/>
@@ -1748,17 +1892,17 @@
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I33" s="6"/>
       <c r="J33" s="7"/>
@@ -1777,17 +1921,17 @@
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="7"/>
@@ -1806,17 +1950,17 @@
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="7"/>
@@ -1830,24 +1974,24 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B36" s="6">
         <v>1</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I36" s="6"/>
       <c r="J36" s="7"/>
@@ -1866,17 +2010,17 @@
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I37" s="6"/>
       <c r="J37" s="7"/>
@@ -1895,17 +2039,17 @@
       </c>
       <c r="C38" s="7"/>
       <c r="D38" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I38" s="6"/>
       <c r="J38" s="7"/>
@@ -1924,17 +2068,17 @@
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="I39" s="6"/>
       <c r="J39" s="7"/>
@@ -1953,17 +2097,17 @@
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I40" s="6"/>
       <c r="J40" s="7"/>
@@ -1982,17 +2126,17 @@
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="I41" s="6"/>
       <c r="J41" s="7"/>
@@ -2004,8 +2148,458 @@
         <v>1</v>
       </c>
     </row>
+    <row r="42" spans="1:13">
+      <c r="A42" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B42" s="6">
+        <v>1</v>
+      </c>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="F42" s="6"/>
+      <c r="G42" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="I42" s="6"/>
+      <c r="J42" s="7"/>
+      <c r="K42" s="7"/>
+      <c r="L42" s="6">
+        <v>1</v>
+      </c>
+      <c r="M42" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="5"/>
+      <c r="B43" s="6">
+        <v>2</v>
+      </c>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="F43" s="6"/>
+      <c r="G43" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="I43" s="6"/>
+      <c r="J43" s="7"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="6">
+        <v>1</v>
+      </c>
+      <c r="M43" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="5"/>
+      <c r="B44" s="6">
+        <v>3</v>
+      </c>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F44" s="6"/>
+      <c r="G44" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="I44" s="6"/>
+      <c r="J44" s="7"/>
+      <c r="K44" s="7"/>
+      <c r="L44" s="6">
+        <v>1</v>
+      </c>
+      <c r="M44" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="5"/>
+      <c r="B45" s="6">
+        <v>4</v>
+      </c>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="F45" s="6"/>
+      <c r="G45" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="I45" s="6"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="6">
+        <v>1</v>
+      </c>
+      <c r="M45" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="5"/>
+      <c r="B46" s="6">
+        <v>5</v>
+      </c>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F46" s="6"/>
+      <c r="G46" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="I46" s="6"/>
+      <c r="J46" s="7"/>
+      <c r="K46" s="7"/>
+      <c r="L46" s="6">
+        <v>1</v>
+      </c>
+      <c r="M46" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13">
+      <c r="A47" s="5"/>
+      <c r="B47" s="6">
+        <v>6</v>
+      </c>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="F47" s="6"/>
+      <c r="G47" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="I47" s="6"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="7"/>
+      <c r="L47" s="6">
+        <v>1</v>
+      </c>
+      <c r="M47" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B48" s="6">
+        <v>1</v>
+      </c>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F48" s="6"/>
+      <c r="G48" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I48" s="6"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="7"/>
+      <c r="L48" s="6">
+        <v>1</v>
+      </c>
+      <c r="M48" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" s="5"/>
+      <c r="B49" s="6">
+        <v>2</v>
+      </c>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="F49" s="6"/>
+      <c r="G49" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="I49" s="6"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="6">
+        <v>1</v>
+      </c>
+      <c r="M49" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13">
+      <c r="A50" s="5"/>
+      <c r="B50" s="6">
+        <v>3</v>
+      </c>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F50" s="6"/>
+      <c r="G50" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I50" s="6"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="6">
+        <v>1</v>
+      </c>
+      <c r="M50" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13">
+      <c r="A51" s="5"/>
+      <c r="B51" s="6">
+        <v>4</v>
+      </c>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F51" s="6"/>
+      <c r="G51" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I51" s="6"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="6">
+        <v>1</v>
+      </c>
+      <c r="M51" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13">
+      <c r="A52" s="5"/>
+      <c r="B52" s="6">
+        <v>5</v>
+      </c>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F52" s="6"/>
+      <c r="G52" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I52" s="6"/>
+      <c r="J52" s="7"/>
+      <c r="K52" s="7"/>
+      <c r="L52" s="6">
+        <v>1</v>
+      </c>
+      <c r="M52" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13">
+      <c r="A53" s="5"/>
+      <c r="B53" s="6">
+        <v>6</v>
+      </c>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F53" s="6"/>
+      <c r="G53" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="I53" s="6"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="7"/>
+      <c r="L53" s="6">
+        <v>1</v>
+      </c>
+      <c r="M53" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13">
+      <c r="A54" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B54" s="6">
+        <v>1</v>
+      </c>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="F54" s="6"/>
+      <c r="G54" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="I54" s="6"/>
+      <c r="J54" s="7"/>
+      <c r="K54" s="7"/>
+      <c r="L54" s="6">
+        <v>1</v>
+      </c>
+      <c r="M54" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13">
+      <c r="A55" s="5"/>
+      <c r="B55" s="6">
+        <v>2</v>
+      </c>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="F55" s="6"/>
+      <c r="G55" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I55" s="6"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="6">
+        <v>1</v>
+      </c>
+      <c r="M55" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13">
+      <c r="A56" s="5"/>
+      <c r="B56" s="6">
+        <v>3</v>
+      </c>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F56" s="6"/>
+      <c r="G56" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I56" s="6"/>
+      <c r="J56" s="7"/>
+      <c r="K56" s="7"/>
+      <c r="L56" s="6">
+        <v>1</v>
+      </c>
+      <c r="M56" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13">
+      <c r="A57" s="5"/>
+    </row>
+    <row r="58" spans="1:13">
+      <c r="A58" s="5"/>
+    </row>
+    <row r="59" spans="1:13">
+      <c r="A59" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="120">
+  <mergeCells count="168">
     <mergeCell ref="A1:K4"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="H5:I5"/>
@@ -2124,6 +2718,54 @@
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="J41:K41"/>
+    <mergeCell ref="A42:A47"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="J44:K44"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="A48:A53"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A54:A59"/>
+    <mergeCell ref="E54:F54"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="J54:K54"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="H55:I55"/>
+    <mergeCell ref="J55:K55"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="J56:K56"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="L4:M4"/>
   </mergeCells>

</xml_diff>

<commit_message>
Updated Readme + file cooperation for easier operation
Now, instead of hardcoding the JSON save.txt and schedule.txt as a data form within json_schedule_parser + xlsx_parser, you can just run the program and it will scan for save.txt and schedule.txt, further expediating the process for creating a meet.
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="170">
   <si>
-    <t>UCD vs UCSC</t>
+    <t>UCD vs UCB</t>
   </si>
   <si>
     <t>Schedule</t>
@@ -37,7 +37,7 @@
     <t>vs.</t>
   </si>
   <si>
-    <t>UCSC</t>
+    <t>UCB</t>
   </si>
   <si>
     <t>Score (Winner First)</t>
@@ -46,52 +46,271 @@
     <t>10:00</t>
   </si>
   <si>
+    <t>WS3</t>
+  </si>
+  <si>
+    <t>vs</t>
+  </si>
+  <si>
+    <t>Chonticha Phanphanit</t>
+  </si>
+  <si>
+    <t>Chaemin Lee</t>
+  </si>
+  <si>
+    <t>MD7</t>
+  </si>
+  <si>
+    <t>Aaron Lim + Bill Wong</t>
+  </si>
+  <si>
+    <t>Jonathan Pan + Jeff Chen</t>
+  </si>
+  <si>
+    <t>WS1</t>
+  </si>
+  <si>
+    <t>Jamie Yip</t>
+  </si>
+  <si>
+    <t>Ziyi Huang</t>
+  </si>
+  <si>
+    <t>WS2</t>
+  </si>
+  <si>
+    <t>Carolyn Suryapermana</t>
+  </si>
+  <si>
+    <t>Emily Qian</t>
+  </si>
+  <si>
+    <t>WD5</t>
+  </si>
+  <si>
+    <t>Winnie Wu + Mallika Chou</t>
+  </si>
+  <si>
+    <t>Anni Zhang + Phoebe Shen</t>
+  </si>
+  <si>
+    <t>MS11</t>
+  </si>
+  <si>
+    <t>Adrian Li</t>
+  </si>
+  <si>
+    <t>Arav Sachdeva</t>
+  </si>
+  <si>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>MS16</t>
+  </si>
+  <si>
+    <t>Booker Brown</t>
+  </si>
+  <si>
+    <t>Kwanghyun Kim</t>
+  </si>
+  <si>
+    <t>MD9</t>
+  </si>
+  <si>
+    <t>Jordon Kwong + Chimnay</t>
+  </si>
+  <si>
+    <t>Kyle Huang + Khai Ho</t>
+  </si>
+  <si>
+    <t>MS15</t>
+  </si>
+  <si>
+    <t>Finn</t>
+  </si>
+  <si>
+    <t>Arion Togelang</t>
+  </si>
+  <si>
+    <t>XD1</t>
+  </si>
+  <si>
+    <t>Leyang Ding + Xin Huang</t>
+  </si>
+  <si>
+    <t>Adam Tay + Angie Huang</t>
+  </si>
+  <si>
+    <t>MD8</t>
+  </si>
+  <si>
+    <t>Daniel Lin + Yawei He</t>
+  </si>
+  <si>
+    <t>Arav Sachdeva + Arun Yadavalli</t>
+  </si>
+  <si>
+    <t>WD3</t>
+  </si>
+  <si>
+    <t>Muyen Liang + Jamie Yip</t>
+  </si>
+  <si>
+    <t>Clarissa Chen + Yuhe Lin</t>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>MD10</t>
+  </si>
+  <si>
+    <t>Michael Salim + Kyle Kimura</t>
+  </si>
+  <si>
+    <t>Howard Huang + Cameron Kato</t>
+  </si>
+  <si>
+    <t>XD7</t>
+  </si>
+  <si>
+    <t>Jonathan Li + Ehong Ng</t>
+  </si>
+  <si>
+    <t>Aarav Rathi + Jane Dong</t>
+  </si>
+  <si>
+    <t>MS1</t>
+  </si>
+  <si>
+    <t>Leyang Ding</t>
+  </si>
+  <si>
+    <t>Adam Tay</t>
+  </si>
+  <si>
+    <t>MD11</t>
+  </si>
+  <si>
+    <t>Ryan Lei + Adrian Luu</t>
+  </si>
+  <si>
+    <t>Zevin Bansal + Vinayak Prathikanti</t>
+  </si>
+  <si>
+    <t>MD13</t>
+  </si>
+  <si>
+    <t>Marc Ethan Saguiped + Donnovan Saelee</t>
+  </si>
+  <si>
+    <t>Wesley Tan + Jansen Mok</t>
+  </si>
+  <si>
+    <t>MS5</t>
+  </si>
+  <si>
+    <t>Jon Moser</t>
+  </si>
+  <si>
+    <t>Zheng Zhou</t>
+  </si>
+  <si>
+    <t>11:30</t>
+  </si>
+  <si>
     <t>WD1</t>
   </si>
   <si>
-    <t>vs</t>
-  </si>
-  <si>
     <t>Xin Huang + Betty Yang</t>
   </si>
   <si>
     <t>Reanne Chan + Ariel Shan</t>
   </si>
   <si>
-    <t>MS1</t>
-  </si>
-  <si>
-    <t>Leyang Ding</t>
-  </si>
-  <si>
-    <t>Adam Tay</t>
-  </si>
-  <si>
-    <t>WS1</t>
-  </si>
-  <si>
-    <t>Jamie Yip</t>
-  </si>
-  <si>
-    <t>Ziyi Huang</t>
-  </si>
-  <si>
-    <t>WD5</t>
-  </si>
-  <si>
-    <t>Winnie Wu + Mallika Chou</t>
-  </si>
-  <si>
-    <t>Anni Zhang + Phoebe Shen</t>
-  </si>
-  <si>
-    <t>WS2</t>
-  </si>
-  <si>
-    <t>Carolyn Suryapermana</t>
-  </si>
-  <si>
-    <t>Emily Qian</t>
+    <t>WD2</t>
+  </si>
+  <si>
+    <t>Kristine Ngo + Erika Lai</t>
+  </si>
+  <si>
+    <t>Kaylee Wang + Kristin Song</t>
+  </si>
+  <si>
+    <t>XD10</t>
+  </si>
+  <si>
+    <t>Richard Huang + Livia Rice</t>
+  </si>
+  <si>
+    <t>Jeff Chen + Stephanie Kuang</t>
+  </si>
+  <si>
+    <t>MS13</t>
+  </si>
+  <si>
+    <t>Michael Salim</t>
+  </si>
+  <si>
+    <t>Joon Choi</t>
+  </si>
+  <si>
+    <t>XD9</t>
+  </si>
+  <si>
+    <t>Adrian Li + Isabella Li</t>
+  </si>
+  <si>
+    <t>Howard Huang + Rosamund Li</t>
+  </si>
+  <si>
+    <t>MS12</t>
+  </si>
+  <si>
+    <t>Kyle Kimura</t>
+  </si>
+  <si>
+    <t>Khai Ho</t>
+  </si>
+  <si>
+    <t>12:00</t>
+  </si>
+  <si>
+    <t>MS14</t>
+  </si>
+  <si>
+    <t>Bill Wong</t>
+  </si>
+  <si>
+    <t>Jack Chu</t>
+  </si>
+  <si>
+    <t>WD4</t>
+  </si>
+  <si>
+    <t>Livia Rice + Isabella Li</t>
+  </si>
+  <si>
+    <t>Angelina Wang + Janina Schieneman</t>
+  </si>
+  <si>
+    <t>XD4</t>
+  </si>
+  <si>
+    <t>Richard Huang + Erika Lai</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Kaylee Wang</t>
+  </si>
+  <si>
+    <t>MS3</t>
+  </si>
+  <si>
+    <t>Mariano Elizondo</t>
+  </si>
+  <si>
+    <t>Brad Chiu</t>
   </si>
   <si>
     <t>MD6</t>
@@ -103,16 +322,187 @@
     <t>Kelsey Lin + Jansen Mok</t>
   </si>
   <si>
-    <t>10:45</t>
-  </si>
-  <si>
-    <t>WD2</t>
-  </si>
-  <si>
-    <t>Kristine Ngo + Erika Lai</t>
-  </si>
-  <si>
-    <t>Kaylee Wang + Kristin Song</t>
+    <t>MS7</t>
+  </si>
+  <si>
+    <t>Sidney Wang</t>
+  </si>
+  <si>
+    <t>Ryan Zhu</t>
+  </si>
+  <si>
+    <t>12:30</t>
+  </si>
+  <si>
+    <t>XD14</t>
+  </si>
+  <si>
+    <t>Jerry Qiu + Suhani Shokeen</t>
+  </si>
+  <si>
+    <t>Haoran Qu + Janina Schieneman</t>
+  </si>
+  <si>
+    <t>MS2</t>
+  </si>
+  <si>
+    <t>Kevin Cuan</t>
+  </si>
+  <si>
+    <t>XD6</t>
+  </si>
+  <si>
+    <t>Adam Dinh + Minh Nguyen</t>
+  </si>
+  <si>
+    <t>Shengkai Jiang + Kristin Song</t>
+  </si>
+  <si>
+    <t>MD1</t>
+  </si>
+  <si>
+    <t>Leyang Ding + Richard Huang</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Jason Arya</t>
+  </si>
+  <si>
+    <t>MS8</t>
+  </si>
+  <si>
+    <t>Jonathan Li</t>
+  </si>
+  <si>
+    <t>MS10</t>
+  </si>
+  <si>
+    <t>Aaron Lim</t>
+  </si>
+  <si>
+    <t>Jake Kim</t>
+  </si>
+  <si>
+    <t>01:00</t>
+  </si>
+  <si>
+    <t>XD13</t>
+  </si>
+  <si>
+    <t>Booker Brown + Chonticha Phanphanit</t>
+  </si>
+  <si>
+    <t>Ajay Sharma + Zinong Wang</t>
+  </si>
+  <si>
+    <t>XD3</t>
+  </si>
+  <si>
+    <t>Kevin Cuan + Iris Lee</t>
+  </si>
+  <si>
+    <t>Ashton Lee + Ashley Huang</t>
+  </si>
+  <si>
+    <t>MD3</t>
+  </si>
+  <si>
+    <t>Jon Moser + Jonathan Li</t>
+  </si>
+  <si>
+    <t>Aarav Rathi + Shengkai Jiang</t>
+  </si>
+  <si>
+    <t>XD11</t>
+  </si>
+  <si>
+    <t>Aaron Lim + Gaby Solei</t>
+  </si>
+  <si>
+    <t>Howie Liang + Angel Yeung</t>
+  </si>
+  <si>
+    <t>MD5</t>
+  </si>
+  <si>
+    <t>Mariano Elizondo + Jerry Qiu</t>
+  </si>
+  <si>
+    <t>Jonathan Pan + Harry Zhang</t>
+  </si>
+  <si>
+    <t>XD2</t>
+  </si>
+  <si>
+    <t>Benson Ngai + Kristine Ngo</t>
+  </si>
+  <si>
+    <t>Patrick Chi + Natalie Chi</t>
+  </si>
+  <si>
+    <t>01:30</t>
+  </si>
+  <si>
+    <t>MD4</t>
+  </si>
+  <si>
+    <t>Sidney Wang + Adrian Luo</t>
+  </si>
+  <si>
+    <t>MS9</t>
+  </si>
+  <si>
+    <t>Sean Tan</t>
+  </si>
+  <si>
+    <t>Arun Yadavalli</t>
+  </si>
+  <si>
+    <t>MD2</t>
+  </si>
+  <si>
+    <t>Benson Ngai + Geoffray Lee</t>
+  </si>
+  <si>
+    <t>Ashley Huang + Natalie Chi</t>
+  </si>
+  <si>
+    <t>XD5</t>
+  </si>
+  <si>
+    <t>Sidney Wang + Betty Yang</t>
+  </si>
+  <si>
+    <t>Ashton Lee + Angie Huang</t>
+  </si>
+  <si>
+    <t>XD12</t>
+  </si>
+  <si>
+    <t>Daniel Lin + Carolyn Surypermana</t>
+  </si>
+  <si>
+    <t>Vinayak Prathikanti + Caitlin Tong</t>
+  </si>
+  <si>
+    <t>MD12</t>
+  </si>
+  <si>
+    <t>Josh Luo + Karthik Villavan</t>
+  </si>
+  <si>
+    <t>Justin Wang + Anton Luu</t>
+  </si>
+  <si>
+    <t>02:00</t>
+  </si>
+  <si>
+    <t>XD8</t>
+  </si>
+  <si>
+    <t>Ryan Lei + Jamie Yip</t>
+  </si>
+  <si>
+    <t>Kelsey Lin + Trinity Nguyen</t>
   </si>
   <si>
     <t>MS4</t>
@@ -121,186 +511,6 @@
     <t>Geoffray Lee</t>
   </si>
   <si>
-    <t>Zheng Zhou</t>
-  </si>
-  <si>
-    <t>WS3</t>
-  </si>
-  <si>
-    <t>Chonticha Phanphanit</t>
-  </si>
-  <si>
-    <t>Chaemin Lee</t>
-  </si>
-  <si>
-    <t>WD3</t>
-  </si>
-  <si>
-    <t>Muyen Liang + Jamie Yip</t>
-  </si>
-  <si>
-    <t>Clarissa Chen + Yuhe Lin</t>
-  </si>
-  <si>
-    <t>MD3</t>
-  </si>
-  <si>
-    <t>Jon Moser + Jonathan Li</t>
-  </si>
-  <si>
-    <t>Aarav Rathi + Shengkai Jiang</t>
-  </si>
-  <si>
-    <t>MD11</t>
-  </si>
-  <si>
-    <t>Ryan Lei + Adrian Luu</t>
-  </si>
-  <si>
-    <t>Zevin Bansal + Vinayak Prathikanti</t>
-  </si>
-  <si>
-    <t>11:30</t>
-  </si>
-  <si>
-    <t>MD4</t>
-  </si>
-  <si>
-    <t>Sidney Wang + Adrian Luo</t>
-  </si>
-  <si>
-    <t>XD8</t>
-  </si>
-  <si>
-    <t>Ryan Lei + Jamie Yip</t>
-  </si>
-  <si>
-    <t>Kelsey Lin + Trinity Nguyen</t>
-  </si>
-  <si>
-    <t>MS8</t>
-  </si>
-  <si>
-    <t>Jonathan Li</t>
-  </si>
-  <si>
-    <t>Ryan Zhu</t>
-  </si>
-  <si>
-    <t>MD9</t>
-  </si>
-  <si>
-    <t>Jordon Kwong + Chimnay</t>
-  </si>
-  <si>
-    <t>Kyle Huang + Khai Ho</t>
-  </si>
-  <si>
-    <t>XD9</t>
-  </si>
-  <si>
-    <t>Adrian Li + Isabella Li</t>
-  </si>
-  <si>
-    <t>Howard Huang + Rosamund Li</t>
-  </si>
-  <si>
-    <t>MD1</t>
-  </si>
-  <si>
-    <t>Leyang Ding + Richard Huang</t>
-  </si>
-  <si>
-    <t>Patrick Chi + Jason Arya</t>
-  </si>
-  <si>
-    <t>12:15</t>
-  </si>
-  <si>
-    <t>XD10</t>
-  </si>
-  <si>
-    <t>Richard Huang + Livia Rice</t>
-  </si>
-  <si>
-    <t>Jeff Chen + Stephanie Kuang</t>
-  </si>
-  <si>
-    <t>MD13</t>
-  </si>
-  <si>
-    <t>Marc Ethan Saguiped + Donnovan Saelee</t>
-  </si>
-  <si>
-    <t>Wesley Tan + Jansen Mok</t>
-  </si>
-  <si>
-    <t>MS14</t>
-  </si>
-  <si>
-    <t>Bill Wong</t>
-  </si>
-  <si>
-    <t>Jack Chu</t>
-  </si>
-  <si>
-    <t>MS11</t>
-  </si>
-  <si>
-    <t>Adrian Li</t>
-  </si>
-  <si>
-    <t>Arav Sachdeva</t>
-  </si>
-  <si>
-    <t>MD2</t>
-  </si>
-  <si>
-    <t>Benson Ngai + Geoffray Lee</t>
-  </si>
-  <si>
-    <t>Ashley Huang + Natalie Chi</t>
-  </si>
-  <si>
-    <t>XD14</t>
-  </si>
-  <si>
-    <t>Jerry Qiu + Suhani Shokeen</t>
-  </si>
-  <si>
-    <t>Haoran Qu + Janina Schieneman</t>
-  </si>
-  <si>
-    <t>01:00</t>
-  </si>
-  <si>
-    <t>MD5</t>
-  </si>
-  <si>
-    <t>Mariano Elizondo + Jerry Qiu</t>
-  </si>
-  <si>
-    <t>Jonathan Pan + Harry Zhang</t>
-  </si>
-  <si>
-    <t>MS15</t>
-  </si>
-  <si>
-    <t>Finn</t>
-  </si>
-  <si>
-    <t>Arion Togelang</t>
-  </si>
-  <si>
-    <t>XD11</t>
-  </si>
-  <si>
-    <t>Aaron Lim + Gaby Solei</t>
-  </si>
-  <si>
-    <t>Howie Liang + Angel Yeung</t>
-  </si>
-  <si>
     <t>MS6</t>
   </si>
   <si>
@@ -308,216 +518,6 @@
   </si>
   <si>
     <t>Jason Arya</t>
-  </si>
-  <si>
-    <t>XD13</t>
-  </si>
-  <si>
-    <t>Booker Brown + Chonticha Phanphanit</t>
-  </si>
-  <si>
-    <t>Ajay Sharma + Zinong Wang</t>
-  </si>
-  <si>
-    <t>XD2</t>
-  </si>
-  <si>
-    <t>Benson Ngai + Kristine Ngo</t>
-  </si>
-  <si>
-    <t>Patrick Chi + Natalie Chi</t>
-  </si>
-  <si>
-    <t>01:45</t>
-  </si>
-  <si>
-    <t>XD7</t>
-  </si>
-  <si>
-    <t>Jonathan Li + Ehong Ng</t>
-  </si>
-  <si>
-    <t>Aarav Rathi + Jane Dong</t>
-  </si>
-  <si>
-    <t>MS16</t>
-  </si>
-  <si>
-    <t>Booker Brown</t>
-  </si>
-  <si>
-    <t>Kwanghyun Kim</t>
-  </si>
-  <si>
-    <t>XD12</t>
-  </si>
-  <si>
-    <t>Daniel Lin + Carolyn Surypermana</t>
-  </si>
-  <si>
-    <t>Vinayak Prathikanti + Caitlin Tong</t>
-  </si>
-  <si>
-    <t>MD12</t>
-  </si>
-  <si>
-    <t>Josh Luo + Karthik Villavan</t>
-  </si>
-  <si>
-    <t>Justin Wang + Anton Luu</t>
-  </si>
-  <si>
-    <t>WD4</t>
-  </si>
-  <si>
-    <t>Livia Rice + Isabella Li</t>
-  </si>
-  <si>
-    <t>Angelina Wang + Janina Schieneman</t>
-  </si>
-  <si>
-    <t>MS13</t>
-  </si>
-  <si>
-    <t>Michael Salim</t>
-  </si>
-  <si>
-    <t>Joon Choi</t>
-  </si>
-  <si>
-    <t>02:30</t>
-  </si>
-  <si>
-    <t>MD7</t>
-  </si>
-  <si>
-    <t>Aaron Lim + Bill Wong</t>
-  </si>
-  <si>
-    <t>Jonathan Pan + Jeff Chen</t>
-  </si>
-  <si>
-    <t>XD6</t>
-  </si>
-  <si>
-    <t>Adam Dinh + Minh Nguyen</t>
-  </si>
-  <si>
-    <t>Shengkai Jiang + Kristin Song</t>
-  </si>
-  <si>
-    <t>XD3</t>
-  </si>
-  <si>
-    <t>Kevin Cuan + Iris Lee</t>
-  </si>
-  <si>
-    <t>Ashton Lee + Ashley Huang</t>
-  </si>
-  <si>
-    <t>XD4</t>
-  </si>
-  <si>
-    <t>Richard Huang + Erika Lai</t>
-  </si>
-  <si>
-    <t>Patrick Chi + Kaylee Wang</t>
-  </si>
-  <si>
-    <t>MD8</t>
-  </si>
-  <si>
-    <t>Daniel Lin + Yawei He</t>
-  </si>
-  <si>
-    <t>Arav Sachdeva + Arun Yadavalli</t>
-  </si>
-  <si>
-    <t>MD10</t>
-  </si>
-  <si>
-    <t>Michael Salim + Kyle Kimura</t>
-  </si>
-  <si>
-    <t>Howard Huang + Cameron Kato</t>
-  </si>
-  <si>
-    <t>03:15</t>
-  </si>
-  <si>
-    <t>MS7</t>
-  </si>
-  <si>
-    <t>Sidney Wang</t>
-  </si>
-  <si>
-    <t>MS10</t>
-  </si>
-  <si>
-    <t>Aaron Lim</t>
-  </si>
-  <si>
-    <t>Jake Kim</t>
-  </si>
-  <si>
-    <t>MS5</t>
-  </si>
-  <si>
-    <t>Jon Moser</t>
-  </si>
-  <si>
-    <t>XD1</t>
-  </si>
-  <si>
-    <t>Leyang Ding + Xin Huang</t>
-  </si>
-  <si>
-    <t>Adam Tay + Angie Huang</t>
-  </si>
-  <si>
-    <t>MS3</t>
-  </si>
-  <si>
-    <t>Mariano Elizondo</t>
-  </si>
-  <si>
-    <t>Brad Chiu</t>
-  </si>
-  <si>
-    <t>MS9</t>
-  </si>
-  <si>
-    <t>Sean Tan</t>
-  </si>
-  <si>
-    <t>Arun Yadavalli</t>
-  </si>
-  <si>
-    <t>04:00</t>
-  </si>
-  <si>
-    <t>MS12</t>
-  </si>
-  <si>
-    <t>Kyle Kimura</t>
-  </si>
-  <si>
-    <t>Khai Ho</t>
-  </si>
-  <si>
-    <t>MS2</t>
-  </si>
-  <si>
-    <t>Kevin Cuan</t>
-  </si>
-  <si>
-    <t>XD5</t>
-  </si>
-  <si>
-    <t>Sidney Wang + Betty Yang</t>
-  </si>
-  <si>
-    <t>Ashton Lee + Angie Huang</t>
   </si>
   <si>
     <t>A-Team Tally</t>
@@ -1030,11 +1030,11 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="4">
-        <f>SUM( L6, L7, L8, L10, L12, L14, L15, L16, L23, L28, L35, L44, L51, L52, L55)</f>
+        <f>SUM( L6, L8, L9, L15, L17, L20, L24, L25, L33, L37, L39, L43, L44, L47, L50)</f>
         <v>0</v>
       </c>
       <c r="M3" s="4">
-        <f>SUM( M6, M7, M8, M10, M12, M14, M15, M16, M23, M28, M35, M44, M51, M52, M55)</f>
+        <f>SUM( M6, M8, M9, M15, M17, M20, M24, M25, M33, M37, M39, M43, M44, M47, M50)</f>
         <v>0</v>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
         <v>11</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" s="7"/>
@@ -1482,17 +1482,17 @@
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="7"/>
@@ -1511,17 +1511,17 @@
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I20" s="6"/>
       <c r="J20" s="7"/>
@@ -1540,17 +1540,17 @@
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="7"/>
@@ -1569,17 +1569,17 @@
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I22" s="6"/>
       <c r="J22" s="7"/>
@@ -1598,17 +1598,17 @@
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="7"/>
@@ -1622,24 +1622,24 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B24" s="6">
         <v>1</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I24" s="6"/>
       <c r="J24" s="7"/>
@@ -1658,17 +1658,17 @@
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I25" s="6"/>
       <c r="J25" s="7"/>
@@ -1687,17 +1687,17 @@
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I26" s="6"/>
       <c r="J26" s="7"/>
@@ -1716,17 +1716,17 @@
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I27" s="6"/>
       <c r="J27" s="7"/>
@@ -1745,17 +1745,17 @@
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I28" s="6"/>
       <c r="J28" s="7"/>
@@ -1774,17 +1774,17 @@
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I29" s="6"/>
       <c r="J29" s="7"/>
@@ -1798,24 +1798,24 @@
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B30" s="6">
         <v>1</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I30" s="6"/>
       <c r="J30" s="7"/>
@@ -1834,17 +1834,17 @@
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="7"/>
@@ -1863,17 +1863,17 @@
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I32" s="6"/>
       <c r="J32" s="7"/>
@@ -1892,17 +1892,17 @@
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I33" s="6"/>
       <c r="J33" s="7"/>
@@ -1921,17 +1921,17 @@
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="7"/>
@@ -1950,17 +1950,17 @@
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="7"/>
@@ -1974,24 +1974,24 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B36" s="6">
         <v>1</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I36" s="6"/>
       <c r="J36" s="7"/>
@@ -2010,17 +2010,17 @@
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="I37" s="6"/>
       <c r="J37" s="7"/>
@@ -2107,7 +2107,7 @@
         <v>11</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="I40" s="6"/>
       <c r="J40" s="7"/>
@@ -2126,17 +2126,17 @@
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>120</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>121</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I41" s="6"/>
       <c r="J41" s="7"/>
@@ -2150,24 +2150,24 @@
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B42" s="6">
         <v>1</v>
       </c>
       <c r="C42" s="7"/>
       <c r="D42" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E42" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="7"/>
@@ -2186,17 +2186,17 @@
       </c>
       <c r="C43" s="7"/>
       <c r="D43" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>128</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I43" s="6"/>
       <c r="J43" s="7"/>
@@ -2215,17 +2215,17 @@
       </c>
       <c r="C44" s="7"/>
       <c r="D44" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I44" s="6"/>
       <c r="J44" s="7"/>
@@ -2244,17 +2244,17 @@
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I45" s="6"/>
       <c r="J45" s="7"/>
@@ -2273,17 +2273,17 @@
       </c>
       <c r="C46" s="7"/>
       <c r="D46" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I46" s="6"/>
       <c r="J46" s="7"/>
@@ -2302,17 +2302,17 @@
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>139</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>140</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I47" s="6"/>
       <c r="J47" s="7"/>
@@ -2326,24 +2326,24 @@
     </row>
     <row r="48" spans="1:13">
       <c r="A48" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B48" s="6">
         <v>1</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>144</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="7"/>
@@ -2362,17 +2362,17 @@
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E49" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I49" s="6"/>
       <c r="J49" s="7"/>
@@ -2391,17 +2391,17 @@
       </c>
       <c r="C50" s="7"/>
       <c r="D50" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="E50" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="5" t="s">
         <v>11</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>35</v>
+        <v>149</v>
       </c>
       <c r="I50" s="6"/>
       <c r="J50" s="7"/>
@@ -2548,7 +2548,7 @@
         <v>11</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>155</v>
+        <v>66</v>
       </c>
       <c r="I55" s="6"/>
       <c r="J55" s="7"/>

</xml_diff>